<commit_message>
Fix #2, updated indicators
</commit_message>
<xml_diff>
--- a/data/FAIR_assessment_template.xlsx
+++ b/data/FAIR_assessment_template.xlsx
@@ -820,7 +820,7 @@
     <t xml:space="preserve">I3-01MA</t>
   </si>
   <si>
-    <t xml:space="preserve">Metadata of archive includes references to other metadata of archive</t>
+    <t xml:space="preserve">Metadata of archive includes references to other metadata</t>
   </si>
   <si>
     <t xml:space="preserve">The indicator is about the way that the archive metadata is connected to other metadata, for example through links to information about organisations, people, places, projects or time periods that are related to the archive that the metadata describes.</t>
@@ -835,7 +835,7 @@
     <t xml:space="preserve">I3-01MM</t>
   </si>
   <si>
-    <t xml:space="preserve">Metadata of model includes references to other metadata of model</t>
+    <t xml:space="preserve">Metadata of model includes references to other metadata</t>
   </si>
   <si>
     <t xml:space="preserve">The indicator is about the way that the model metadata is connected to other metadata, for example through links to information about organisations, people, places, projects or time periods that are related to the model that the metadata describes.</t>
@@ -4058,14 +4058,14 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J2:J85" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J2:J85" type="list">
       <formula1>"1,0.5,0,NA"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>